<commit_message>
docs: polish report contents for japanese delivery
</commit_message>
<xml_diff>
--- a/artifacts/reports/testcases/TC-IT-API-01_VoIPWebAPI結合テスト/TC-IT-API-01_VoIPWebAPI結合テストケース.xlsx
+++ b/artifacts/reports/testcases/TC-IT-API-01_VoIPWebAPI結合テスト/TC-IT-API-01_VoIPWebAPI結合テストケース.xlsx
@@ -7631,7 +7631,7 @@
       <c r="I55" s="6" t="n"/>
       <c r="J55" s="62" t="inlineStr">
         <is>
-          <t>Nhập sai mã OTP 5 lần liên tiếp</t>
+          <t>OTPを5回連続で誤入力する</t>
         </is>
       </c>
       <c r="K55" s="5" t="n"/>
@@ -7650,7 +7650,7 @@
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="62" t="inlineStr">
         <is>
-          <t>① 対象機能「Nhập sai mã OTP 5 lần liên tiếp」に対応するAPIを呼び出す。
+          <t>① 対象機能「OTPを5回連続で誤入力する」に対応するAPIを呼び出す。
 ② 必要な認証情報、入力データ、CSVファイルまたはスタブ応答を準備する。
 ③ HTTPステータス、レスポンス内容、必要なDB更新を確認する。</t>
         </is>

</xml_diff>

<commit_message>
docs: restore testcase environment labels
</commit_message>
<xml_diff>
--- a/artifacts/reports/testcases/TC-IT-API-01_VoIPWebAPI結合テスト/TC-IT-API-01_VoIPWebAPI結合テストケース.xlsx
+++ b/artifacts/reports/testcases/TC-IT-API-01_VoIPWebAPI結合テスト/TC-IT-API-01_VoIPWebAPI結合テストケース.xlsx
@@ -2403,7 +2403,7 @@
       <c r="AF5" s="29" t="n"/>
       <c r="AG5" s="34" t="inlineStr">
         <is>
-          <t>テスト結果 - 第1回</t>
+          <t>テスト結果 - 第1回（ローカル）</t>
         </is>
       </c>
       <c r="AH5" s="31" t="n"/>
@@ -2421,7 +2421,7 @@
       <c r="AT5" s="32" t="n"/>
       <c r="AU5" s="34" t="inlineStr">
         <is>
-          <t>テスト結果 - 第2回</t>
+          <t>テスト結果 - 第2回（ローカル）</t>
         </is>
       </c>
       <c r="AV5" s="31" t="n"/>

</xml_diff>